<commit_message>
[Flowguard-7] Added UI + updated pipeline.
</commit_message>
<xml_diff>
--- a/reports/latest/demo_showcase/02_icedid_shifted/top_incidents.xlsx
+++ b/reports/latest/demo_showcase/02_icedid_shifted/top_incidents.xlsx
@@ -525,7 +525,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -556,7 +556,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.6с, объём≈9733 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.6с, объём ~9733 Б</t>
         </is>
       </c>
     </row>
@@ -587,7 +587,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈10099 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~10099 Б</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈5.1с, объём≈12488 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~5.1с, объём ~12488 Б</t>
         </is>
       </c>
     </row>
@@ -711,7 +711,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈1.6с, объём≈9626 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~1.6с, объём ~9626 Б</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈60.4с, объём≈12139 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~60.4с, объём ~12139 Б</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.7с, объём≈8534 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.7с, объём ~8534 Б</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=3, длительность≈0.6с, объём≈8900 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=3, длительность ~0.6с, объём ~8900 Б</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈60.3с, объём≈11817 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~60.3с, объём ~11817 Б</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈8533 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~8533 Б</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈14.2с, объём≈19008 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~14.2с, объём ~19008 Б</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈5.1с, объём≈10965 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~5.1с, объём ~10965 Б</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~61.4с</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Короткая TLS-сессия</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Короткое TLS-соединение: длительность≈0.55с, объём≈9979 Б, пакеты≈31</t>
+          <t>Короткое TLS-соединение без явного паттерна: длительность ~0.55с, объём ~9979 Б</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.7с, объём≈11347 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.7с, объём ~11347 Б</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈8715 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~8715 Б</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈8533 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~8533 Б</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.3с, объём≈10247 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.3с, объём ~10247 Б</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈8586 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~8586 Б</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈2.7с, объём≈8644 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~2.7с, объём ~8644 Б</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈8537 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~8537 Б</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.5с, объём≈22735 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.5с, объём ~22735 Б</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.4с, объём≈9913 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.4с, объём ~9913 Б</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=3, длительность≈5.4с, объём≈18180 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=3, длительность ~5.4с, объём ~18180 Б</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~109.9с</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈1.6с, объём≈6663 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~1.6с, объём ~6663 Б</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~109.9с</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~106.9с</t>
         </is>
       </c>
     </row>
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Короткая TLS-сессия</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Короткое TLS-соединение: длительность≈0.59с, объём≈7348 Б, пакеты≈20</t>
+          <t>Короткое TLS-соединение без явного паттерна: длительность ~0.59с, объём ~7348 Б</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=3, длительность≈20.5с, объём≈8171 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=3, длительность ~20.5с, объём ~8171 Б</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.6с, объём≈17942 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.6с, объём ~17942 Б</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.3с, объём≈6966 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.3с, объём ~6966 Б</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~0.4с</t>
         </is>
       </c>
     </row>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~0.8с</t>
         </is>
       </c>
     </row>
@@ -2571,7 +2571,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈2.5с, объём≈22190 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~2.5с, объём ~22190 Б</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~65.0с</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~0.2с</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈1.3с, объём≈58617 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~1.3с, объём ~58617 Б</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.8с, объём≈7295 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.8с, объём ~7295 Б</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2881,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=2, длительность≈0.3с, объём≈42630 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=2, длительность ~0.3с, объём ~42630 Б</t>
         </is>
       </c>
     </row>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈0.3с, объём≈9438 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~0.3с, объём ~9438 Б</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=2, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 2, длительность ~68.4с</t>
         </is>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~0.3с</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=1, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 1, длительность ~0.3с</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=62, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 62, длительность ~67.3с</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3253,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50884 (вне [443, 8443, 9443]): flows=1, длительность≈0.1с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50884; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.1с</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈19.9с, объём≈11116 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~19.9с, объём ~11116 Б</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=2, длительность≈11.4с, объём≈217974 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=2, длительность ~11.4с, объём ~217974 Б</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=5, длительность≈1.6с, объём≈6684 Б, ALPN=2 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=5, длительность ~1.6с, объём ~6684 Б</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=5, длительность≈0.3с, объём≈3117 Б, ALPN=2 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=5, длительность ~0.3с, объём ~3117 Б</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=2, длительность≈22.3с, объём≈24869 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=2, длительность ~22.3с, объём ~24869 Б</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>TLS без SNI</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>TLS-соединения без Server Name Indication: flows=2, no_sni_ratio=50%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: отсутствует SNI у 50% сессий; не-браузерный ALPN. Сессий: 2, длительность ~0.2с</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>TLS без SNI</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>TLS-соединения без Server Name Indication: flows=2, no_sni_ratio=50%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: отсутствует SNI у 50% сессий; не-браузерный ALPN. Сессий: 2, длительность ~0.2с</t>
         </is>
       </c>
     </row>
@@ -3749,7 +3749,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>TLS без SNI</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>TLS-соединения без Server Name Indication: flows=2, no_sni_ratio=50%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: отсутствует SNI у 50% сессий; не-браузерный ALPN. Сессий: 2, длительность ~0.4с</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈24.1с, объём≈10759 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~24.1с, объём ~10759 Б</t>
         </is>
       </c>
     </row>
@@ -3873,7 +3873,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈19.2с, объём≈11783 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~19.2с, объём ~11783 Б</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈19.9с, объём≈9028 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~19.9с, объём ~9028 Б</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈23.9с, объём≈24064 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~23.9с, объём ~24064 Б</t>
         </is>
       </c>
     </row>
@@ -4059,7 +4059,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈21.7с, объём≈172240 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~21.7с, объём ~172240 Б</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>TLS без ALPN / нестандартный ALPN</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Не-браузерный TLS-стек: flows=76, empty_alpn=100%, common_alpn=100%</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: не-браузерный ALPN. Сессий: 76, длительность ~1.0с</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=2, длительность≈19.9с, объём≈42097 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=2, длительность ~19.9с, объём ~42097 Б</t>
         </is>
       </c>
     </row>
@@ -4245,7 +4245,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -4276,7 +4276,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=2, длительность≈12.3с, объём≈11086 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=2, длительность ~12.3с, объём ~11086 Б</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4307,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>TLS-аномалия без явного паттерна</t>
+          <t>Неклассифицированная аномалия</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>TLS-соединение помечено моделью как аномалия: flows=2, длительность≈12.3с, объём≈10256 Б, ALPN=1 вариант(ов)</t>
+          <t>TLS-соединение помечено моделью как аномалия: сессий=2, длительность ~12.3с, объём ~10256 Б</t>
         </is>
       </c>
     </row>
@@ -4369,7 +4369,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -4400,7 +4400,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈3</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~3</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Выраженное преобладание входящего трафика: s2c=4606686 Б, c2s=98588 Б</t>
+          <t>Преобладание входящего трафика: вх=4606686 Б, исх=98588 Б</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4555,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4617,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -4772,7 +4772,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4803,7 +4803,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4865,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -4989,7 +4989,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Активный клиент с множеством TLS-соединений</t>
+          <t>Активный TLS-клиент</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>Клиент показывает атипичный паттерн: 240 аномальных flows к 66 серверам. Данное соединение: длительность≈8.5с, объём≈6729 Б, ALPN=1</t>
+          <t>Клиент проявляет атипично широкую активность: 240 аномальных сессий к 66 серверам. Данная сессия: длительность ~8.5с, объём ~6729 Б</t>
         </is>
       </c>
     </row>
@@ -5113,7 +5113,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50867 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50867; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5237,7 +5237,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -5392,7 +5392,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5733,7 +5733,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -5826,7 +5826,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50834 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50834; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50845 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50845; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -5950,7 +5950,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50915 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50915; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50924 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50924; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6043,7 +6043,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50928 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50928; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6105,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -6136,7 +6136,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50929 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50929; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -6198,7 +6198,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 51052 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 51052; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6229,7 +6229,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -6260,7 +6260,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 51053 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 51053; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 51058 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 51058; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6353,7 +6353,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -6384,7 +6384,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 51079 (вне [443, 8443, 9443]): flows=1, длительность≈0.0с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 51079; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.0с</t>
         </is>
       </c>
     </row>
@@ -6415,7 +6415,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>TLS на нестандартном порту</t>
+          <t>Подозрительный TLS-профиль</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>TLS-соединение на порту 50876 (вне [443, 8443, 9443]): flows=1, длительность≈0.4с</t>
+          <t>TLS-профиль содержит признаки не-браузерного стека: нестандартный порт 50876; отсутствует SNI у 100% сессий; не-браузерный ALPN. Сессий: 1, длительность ~0.4с</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -6570,7 +6570,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Сканирование портов (fan-out)</t>
+          <t>Веерное сканирование портов</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>Клиент сканирует 40 портов на 1 серверах: flow_duration≈0.00с, packets≈2</t>
+          <t>Клиент сканирует 40 портов на 1 серверах: длительность ~0.00с, пакетов ~2</t>
         </is>
       </c>
     </row>

</xml_diff>